<commit_message>
Ranking: gasto total e carga de tributos federais (Tesouro, % do PIB)
- adapters/tesouro.js (tesouro@2): da aba 2.1-A do RTN lê também a
  despesa total (linha 4) e os tributos federais (1.1 + 1.2 + 1.3, com
  proteção contra contar incentivos duas vezes); linha ausente gera erro
  com os rótulos encontrados.
- Ambos no ranking oficial com "menor é melhor" (régua declarada na
  metodologia, peso ajustável), cobrindo 1997 em diante.
- Despesa do FMI fica como visão do governo geral, para consulta.
- 65 testes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5VsgUVmUFMniSDuBdCSqB
</commit_message>
<xml_diff>
--- a/test/fixtures/rtn-mini.xlsx
+++ b/test/fixtures/rtn-mini.xlsx
@@ -26,6 +26,18 @@
     <t xml:space="preserve">1. RECEITA TOTAL 1/</t>
   </si>
   <si>
+    <t xml:space="preserve">1.1 - Receita Administrada pela RFB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2 - Incentivos Fiscais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.3 - Arrecadação Líquida para o RGPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. DESPESA TOTAL 2/</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.2  Pessoal e Encargos Sociais</t>
   </si>
   <si>
@@ -248,9 +260,377 @@
         <v>0.2</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>0.12</v>
+      </c>
+      <c r="C7">
+        <v>0.12</v>
+      </c>
+      <c r="D7">
+        <v>0.12</v>
+      </c>
+      <c r="E7">
+        <v>0.12</v>
+      </c>
+      <c r="F7">
+        <v>0.12</v>
+      </c>
+      <c r="G7">
+        <v>0.12</v>
+      </c>
+      <c r="H7">
+        <v>0.12</v>
+      </c>
+      <c r="I7">
+        <v>0.12</v>
+      </c>
+      <c r="J7">
+        <v>0.12</v>
+      </c>
+      <c r="K7">
+        <v>0.12</v>
+      </c>
+      <c r="L7">
+        <v>0.12</v>
+      </c>
+      <c r="M7">
+        <v>0.12</v>
+      </c>
+      <c r="N7">
+        <v>0.12</v>
+      </c>
+      <c r="O7">
+        <v>0.12</v>
+      </c>
+      <c r="P7">
+        <v>0.12</v>
+      </c>
+      <c r="Q7">
+        <v>0.12</v>
+      </c>
+      <c r="R7">
+        <v>0.12</v>
+      </c>
+      <c r="S7">
+        <v>0.12</v>
+      </c>
+      <c r="T7">
+        <v>0.12</v>
+      </c>
+      <c r="U7">
+        <v>0.12</v>
+      </c>
+      <c r="V7">
+        <v>0.12</v>
+      </c>
+      <c r="W7">
+        <v>0.12</v>
+      </c>
+      <c r="X7">
+        <v>0.12</v>
+      </c>
+      <c r="Y7">
+        <v>0.12</v>
+      </c>
+      <c r="Z7">
+        <v>0.12</v>
+      </c>
+      <c r="AA7">
+        <v>0.12</v>
+      </c>
+      <c r="AB7">
+        <v>0.12</v>
+      </c>
+      <c r="AC7">
+        <v>0.12</v>
+      </c>
+      <c r="AD7">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>-0.001</v>
+      </c>
+      <c r="C8">
+        <v>-0.001</v>
+      </c>
+      <c r="D8">
+        <v>-0.001</v>
+      </c>
+      <c r="E8">
+        <v>-0.001</v>
+      </c>
+      <c r="F8">
+        <v>-0.001</v>
+      </c>
+      <c r="G8">
+        <v>-0.001</v>
+      </c>
+      <c r="H8">
+        <v>-0.001</v>
+      </c>
+      <c r="I8">
+        <v>-0.001</v>
+      </c>
+      <c r="J8">
+        <v>-0.001</v>
+      </c>
+      <c r="K8">
+        <v>-0.001</v>
+      </c>
+      <c r="L8">
+        <v>-0.001</v>
+      </c>
+      <c r="M8">
+        <v>-0.001</v>
+      </c>
+      <c r="N8">
+        <v>-0.001</v>
+      </c>
+      <c r="O8">
+        <v>-0.001</v>
+      </c>
+      <c r="P8">
+        <v>-0.001</v>
+      </c>
+      <c r="Q8">
+        <v>-0.001</v>
+      </c>
+      <c r="R8">
+        <v>-0.001</v>
+      </c>
+      <c r="S8">
+        <v>-0.001</v>
+      </c>
+      <c r="T8">
+        <v>-0.001</v>
+      </c>
+      <c r="U8">
+        <v>-0.001</v>
+      </c>
+      <c r="V8">
+        <v>-0.001</v>
+      </c>
+      <c r="W8">
+        <v>-0.001</v>
+      </c>
+      <c r="X8">
+        <v>-0.001</v>
+      </c>
+      <c r="Y8">
+        <v>-0.001</v>
+      </c>
+      <c r="Z8">
+        <v>-0.001</v>
+      </c>
+      <c r="AA8">
+        <v>-0.001</v>
+      </c>
+      <c r="AB8">
+        <v>-0.001</v>
+      </c>
+      <c r="AC8">
+        <v>-0.001</v>
+      </c>
+      <c r="AD8">
+        <v>-0.001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>0.05</v>
+      </c>
+      <c r="C9">
+        <v>0.05</v>
+      </c>
+      <c r="D9">
+        <v>0.05</v>
+      </c>
+      <c r="E9">
+        <v>0.05</v>
+      </c>
+      <c r="F9">
+        <v>0.05</v>
+      </c>
+      <c r="G9">
+        <v>0.05</v>
+      </c>
+      <c r="H9">
+        <v>0.05</v>
+      </c>
+      <c r="I9">
+        <v>0.05</v>
+      </c>
+      <c r="J9">
+        <v>0.05</v>
+      </c>
+      <c r="K9">
+        <v>0.05</v>
+      </c>
+      <c r="L9">
+        <v>0.05</v>
+      </c>
+      <c r="M9">
+        <v>0.05</v>
+      </c>
+      <c r="N9">
+        <v>0.05</v>
+      </c>
+      <c r="O9">
+        <v>0.05</v>
+      </c>
+      <c r="P9">
+        <v>0.05</v>
+      </c>
+      <c r="Q9">
+        <v>0.05</v>
+      </c>
+      <c r="R9">
+        <v>0.05</v>
+      </c>
+      <c r="S9">
+        <v>0.05</v>
+      </c>
+      <c r="T9">
+        <v>0.05</v>
+      </c>
+      <c r="U9">
+        <v>0.05</v>
+      </c>
+      <c r="V9">
+        <v>0.05</v>
+      </c>
+      <c r="W9">
+        <v>0.05</v>
+      </c>
+      <c r="X9">
+        <v>0.05</v>
+      </c>
+      <c r="Y9">
+        <v>0.05</v>
+      </c>
+      <c r="Z9">
+        <v>0.05</v>
+      </c>
+      <c r="AA9">
+        <v>0.05</v>
+      </c>
+      <c r="AB9">
+        <v>0.05</v>
+      </c>
+      <c r="AC9">
+        <v>0.05</v>
+      </c>
+      <c r="AD9">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30">
+        <v>0.18</v>
+      </c>
+      <c r="C30">
+        <v>0.18</v>
+      </c>
+      <c r="D30">
+        <v>0.18</v>
+      </c>
+      <c r="E30">
+        <v>0.18</v>
+      </c>
+      <c r="F30">
+        <v>0.18</v>
+      </c>
+      <c r="G30">
+        <v>0.18</v>
+      </c>
+      <c r="H30">
+        <v>0.18</v>
+      </c>
+      <c r="I30">
+        <v>0.18</v>
+      </c>
+      <c r="J30">
+        <v>0.18</v>
+      </c>
+      <c r="K30">
+        <v>0.18</v>
+      </c>
+      <c r="L30">
+        <v>0.18</v>
+      </c>
+      <c r="M30">
+        <v>0.18</v>
+      </c>
+      <c r="N30">
+        <v>0.18</v>
+      </c>
+      <c r="O30">
+        <v>0.18</v>
+      </c>
+      <c r="P30">
+        <v>0.18</v>
+      </c>
+      <c r="Q30">
+        <v>0.18</v>
+      </c>
+      <c r="R30">
+        <v>0.18</v>
+      </c>
+      <c r="S30">
+        <v>0.18</v>
+      </c>
+      <c r="T30">
+        <v>0.18</v>
+      </c>
+      <c r="U30">
+        <v>0.18</v>
+      </c>
+      <c r="V30">
+        <v>0.18</v>
+      </c>
+      <c r="W30">
+        <v>0.18</v>
+      </c>
+      <c r="X30">
+        <v>0.18</v>
+      </c>
+      <c r="Y30">
+        <v>0.18</v>
+      </c>
+      <c r="Z30">
+        <v>0.18</v>
+      </c>
+      <c r="AA30">
+        <v>0.18</v>
+      </c>
+      <c r="AB30">
+        <v>0.18</v>
+      </c>
+      <c r="AC30">
+        <v>0.18</v>
+      </c>
+      <c r="AD30">
+        <v>0.18</v>
+      </c>
+    </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B41">
         <v>0.045</v>
@@ -342,7 +722,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B78">
         <v>1000000.0</v>

</xml_diff>

<commit_message>
Cobertura fiscal do FHC: resultado primário do governo central pelo Tesouro
- tesouro@3: lê do RTN (aba 2.1-A, desde 1997) o resultado primário do
  governo central (linha 5, ou receita líquida − despesa total) e os
  juros nominais (linha 9, opcional, guardados como custo).
- Ranking usa o primário do Tesouro: mesmo perímetro dos indicadores de
  gasto, tributos e pessoal, e cobre 6 de 8 anos do FHC (FMI só 2001+).
- Contexto: herança fiscal pelo Tesouro, com FMI como reserva.
- 70 testes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5VsgUVmUFMniSDuBdCSqB
</commit_message>
<xml_diff>
--- a/test/fixtures/rtn-mini.xlsx
+++ b/test/fixtures/rtn-mini.xlsx
@@ -43,6 +43,12 @@
   <si>
     <t xml:space="preserve"> PIB Nominal (R$ Milhões)</t>
   </si>
+  <si>
+    <t xml:space="preserve">5. RESULTADO PRIMÁRIO DO GOV. CENTRAL (3-4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. JUROS NOMINAIS</t>
+  </si>
 </sst>
 </file>
 
@@ -720,6 +726,190 @@
         <v>0.031</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>11</v>
+      </c>
+      <c r="B60">
+        <v>0.02</v>
+      </c>
+      <c r="C60">
+        <v>0.02</v>
+      </c>
+      <c r="D60">
+        <v>0.02</v>
+      </c>
+      <c r="E60">
+        <v>0.02</v>
+      </c>
+      <c r="F60">
+        <v>0.02</v>
+      </c>
+      <c r="G60">
+        <v>0.02</v>
+      </c>
+      <c r="H60">
+        <v>0.02</v>
+      </c>
+      <c r="I60">
+        <v>0.02</v>
+      </c>
+      <c r="J60">
+        <v>0.02</v>
+      </c>
+      <c r="K60">
+        <v>0.02</v>
+      </c>
+      <c r="L60">
+        <v>-0.01</v>
+      </c>
+      <c r="M60">
+        <v>-0.01</v>
+      </c>
+      <c r="N60">
+        <v>-0.01</v>
+      </c>
+      <c r="O60">
+        <v>-0.01</v>
+      </c>
+      <c r="P60">
+        <v>-0.01</v>
+      </c>
+      <c r="Q60">
+        <v>-0.01</v>
+      </c>
+      <c r="R60">
+        <v>-0.01</v>
+      </c>
+      <c r="S60">
+        <v>-0.01</v>
+      </c>
+      <c r="T60">
+        <v>-0.01</v>
+      </c>
+      <c r="U60">
+        <v>-0.01</v>
+      </c>
+      <c r="V60">
+        <v>-0.01</v>
+      </c>
+      <c r="W60">
+        <v>-0.01</v>
+      </c>
+      <c r="X60">
+        <v>-0.01</v>
+      </c>
+      <c r="Y60">
+        <v>-0.01</v>
+      </c>
+      <c r="Z60">
+        <v>-0.01</v>
+      </c>
+      <c r="AA60">
+        <v>-0.01</v>
+      </c>
+      <c r="AB60">
+        <v>-0.01</v>
+      </c>
+      <c r="AC60">
+        <v>-0.01</v>
+      </c>
+      <c r="AD60">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>12</v>
+      </c>
+      <c r="B70">
+        <v>-0.05</v>
+      </c>
+      <c r="C70">
+        <v>-0.05</v>
+      </c>
+      <c r="D70">
+        <v>-0.05</v>
+      </c>
+      <c r="E70">
+        <v>-0.05</v>
+      </c>
+      <c r="F70">
+        <v>-0.05</v>
+      </c>
+      <c r="G70">
+        <v>-0.05</v>
+      </c>
+      <c r="H70">
+        <v>-0.05</v>
+      </c>
+      <c r="I70">
+        <v>-0.05</v>
+      </c>
+      <c r="J70">
+        <v>-0.05</v>
+      </c>
+      <c r="K70">
+        <v>-0.05</v>
+      </c>
+      <c r="L70">
+        <v>-0.05</v>
+      </c>
+      <c r="M70">
+        <v>-0.05</v>
+      </c>
+      <c r="N70">
+        <v>-0.05</v>
+      </c>
+      <c r="O70">
+        <v>-0.05</v>
+      </c>
+      <c r="P70">
+        <v>-0.05</v>
+      </c>
+      <c r="Q70">
+        <v>-0.05</v>
+      </c>
+      <c r="R70">
+        <v>-0.05</v>
+      </c>
+      <c r="S70">
+        <v>-0.05</v>
+      </c>
+      <c r="T70">
+        <v>-0.05</v>
+      </c>
+      <c r="U70">
+        <v>-0.05</v>
+      </c>
+      <c r="V70">
+        <v>-0.05</v>
+      </c>
+      <c r="W70">
+        <v>-0.05</v>
+      </c>
+      <c r="X70">
+        <v>-0.05</v>
+      </c>
+      <c r="Y70">
+        <v>-0.05</v>
+      </c>
+      <c r="Z70">
+        <v>-0.05</v>
+      </c>
+      <c r="AA70">
+        <v>-0.05</v>
+      </c>
+      <c r="AB70">
+        <v>-0.05</v>
+      </c>
+      <c r="AC70">
+        <v>-0.05</v>
+      </c>
+      <c r="AD70">
+        <v>-0.05</v>
+      </c>
+    </row>
     <row r="78">
       <c r="A78" t="s">
         <v>10</v>

</xml_diff>